<commit_message>
feat: contact submission, language api.
</commit_message>
<xml_diff>
--- a/public/templates/contact-submissions.xlsx
+++ b/public/templates/contact-submissions.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="19">
   <si>
     <t>name</t>
   </si>
@@ -26,7 +26,10 @@
     <t>phone</t>
   </si>
   <si>
-    <t>place</t>
+    <t>country</t>
+  </si>
+  <si>
+    <t>company</t>
   </si>
   <si>
     <t>subject</t>
@@ -41,7 +44,10 @@
     <t>john@example.com</t>
   </si>
   <si>
-    <t>New York</t>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>Example Corp</t>
   </si>
   <si>
     <t>Product Inquiry</t>
@@ -56,10 +62,10 @@
     <t>jane@example.com</t>
   </si>
   <si>
-    <t>+0987654321</t>
-  </si>
-  <si>
-    <t>London</t>
+    <t>United Kingdom</t>
+  </si>
+  <si>
+    <t>Tech Ltd</t>
   </si>
   <si>
     <t>Support Request</t>
@@ -405,10 +411,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -427,45 +433,54 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2">
         <v>1234567890</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="C3">
+        <v>44987654321</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>